<commit_message>
Updated code to run from root of DefaultData.
Updaed Diagnostic editor values
</commit_message>
<xml_diff>
--- a/SourceData/tuberculosis/TBDiagnosticEditorDefaults2024.xlsx
+++ b/SourceData/tuberculosis/TBDiagnosticEditorDefaults2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proj\Spectrum\DefaultData\SourceData\tuberculosis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RachelSanders\Avenir Health Dropbox\Rachel Sanders\Files\TB\TB online\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D6196E7-8F6C-4AE8-A27E-09271D1094F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B04C70E-71E7-403C-BED2-5FC36EEEB66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="885" firstSheet="10" activeTab="11" xr2:uid="{FBBD4383-2B44-42EB-8787-C2351F8B2CAE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="885" firstSheet="8" activeTab="18" xr2:uid="{FBBD4383-2B44-42EB-8787-C2351F8B2CAE}"/>
   </bookViews>
   <sheets>
     <sheet name="PulmTB HIVNeg Child" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="173">
   <si>
     <t>mWRD [all samples] and Moderate complexity automated NAAT [MC-aNAAT][only on sputum samples][choice]</t>
   </si>
@@ -690,6 +690,18 @@
   <si>
     <t>LC-aNAAT_LF-LAM</t>
   </si>
+  <si>
+    <t>NPOC_NAAT_sputum</t>
+  </si>
+  <si>
+    <t>NPOC_NAAT_swab</t>
+  </si>
+  <si>
+    <t>NPOC-NAAT on sputum</t>
+  </si>
+  <si>
+    <t>NPOC-NAAT on tongue swab</t>
+  </si>
 </sst>
 </file>
 
@@ -699,7 +711,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -800,6 +812,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Inherit"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -867,7 +884,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -933,6 +950,10 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1248,13 +1269,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AF96998-75A9-4731-A9E7-1B9F9C434A94}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="101.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -1262,7 +1283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -1282,7 +1303,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1290,7 +1311,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -1302,15 +1323,15 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.64</v>
       </c>
       <c r="F4">
-        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -1322,15 +1343,15 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.75</v>
       </c>
       <c r="F5">
-        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -1342,15 +1363,15 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <f>VLOOKUP(B6,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B6,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>1</v>
       </c>
       <c r="F6">
-        <f>VLOOKUP(B6,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <f>VLOOKUP(B6,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -1362,15 +1383,15 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <f>VLOOKUP(B7,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B7,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>1</v>
       </c>
       <c r="F7">
-        <f>VLOOKUP(B7,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <f>VLOOKUP(B7,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1378,7 +1399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -1390,15 +1411,15 @@
         <v>1</v>
       </c>
       <c r="E9">
-        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.65</v>
       </c>
       <c r="F9">
-        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -1410,15 +1431,15 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.753</v>
       </c>
       <c r="F10">
-        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -1430,15 +1451,15 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.73</v>
       </c>
       <c r="F11">
-        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -1450,15 +1471,15 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.8</v>
       </c>
       <c r="F12">
-        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -1470,15 +1491,15 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.84099999999999997</v>
       </c>
       <c r="F13">
-        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -1490,15 +1511,15 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.96</v>
       </c>
       <c r="F14">
-        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -1510,87 +1531,118 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.93</v>
       </c>
       <c r="F15">
-        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
       <c r="C16">
-        <f>VLOOKUP(B16, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B16, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>14</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.91</v>
       </c>
       <c r="F16">
-        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
       <c r="C17">
-        <f>VLOOKUP(B17, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B17, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>27</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.93</v>
       </c>
       <c r="F17">
-        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>161</v>
       </c>
       <c r="C18">
+        <f>VLOOKUP(B18, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>45</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18">
-        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,4,FALSE)</f>
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
         <v>0.79900000000000004</v>
       </c>
       <c r="F18">
-        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
         <v>0.93400000000000005</v>
       </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="B27" s="29"/>
+    </row>
+    <row r="29" spans="2:6">
+      <c r="B29" s="29"/>
+    </row>
+    <row r="31" spans="2:6">
+      <c r="B31" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76A64F5A-7933-4AC4-AD1C-26C900B13748}">
-  <dimension ref="A1:G27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="51.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>56</v>
       </c>
@@ -1598,7 +1650,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -1618,7 +1670,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1626,7 +1678,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -1646,7 +1698,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -1666,7 +1718,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -1684,7 +1736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -1702,7 +1754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -1710,7 +1762,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>39</v>
       </c>
@@ -1730,7 +1782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>40</v>
       </c>
@@ -1750,7 +1802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>41</v>
       </c>
@@ -1770,7 +1822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>42</v>
       </c>
@@ -1790,7 +1842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>43</v>
       </c>
@@ -1810,7 +1862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>44</v>
       </c>
@@ -1830,7 +1882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>45</v>
       </c>
@@ -1850,7 +1902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>46</v>
       </c>
@@ -1870,7 +1922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="B17" t="s">
         <v>47</v>
       </c>
@@ -1890,7 +1942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="B18" t="s">
         <v>48</v>
       </c>
@@ -1910,7 +1962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="B19" t="s">
         <v>49</v>
       </c>
@@ -1930,7 +1982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="B20" t="s">
         <v>50</v>
       </c>
@@ -1950,7 +2002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="B21" t="s">
         <v>51</v>
       </c>
@@ -1970,7 +2022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="B22" t="s">
         <v>52</v>
       </c>
@@ -1990,7 +2042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="B23" t="s">
         <v>53</v>
       </c>
@@ -2010,7 +2062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -2018,7 +2070,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7">
       <c r="B25" t="s">
         <v>1</v>
       </c>
@@ -2038,7 +2090,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7">
       <c r="B26" t="s">
         <v>2</v>
       </c>
@@ -2058,7 +2110,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7">
       <c r="B27" t="s">
         <v>160</v>
       </c>
@@ -2075,6 +2127,46 @@
       <c r="F27">
         <f>VLOOKUP(B27,DiagnosisSensAndSpec!$E$2:$G$48,3,FALSE)</f>
         <v>0.89400000000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="B28" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C28">
+        <f>VLOOKUP(B28, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <f>VLOOKUP(B28,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F28">
+        <f>VLOOKUP(B28,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="B29" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C29">
+        <f>VLOOKUP(B29, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>48</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <f>VLOOKUP(B29,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="F29">
+        <f>VLOOKUP(B29,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.99199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2084,13 +2176,13 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C37266C7-EB10-4E6B-A67D-5B083FC0407A}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="51.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>136</v>
       </c>
@@ -2098,7 +2190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -2118,7 +2210,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -2126,7 +2218,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -2146,7 +2238,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -2166,7 +2258,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -2186,7 +2278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -2206,7 +2298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -2214,7 +2306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2234,7 +2326,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -2254,7 +2346,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -2274,7 +2366,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -2294,7 +2386,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2314,7 +2406,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -2334,7 +2426,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -2354,7 +2446,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -2374,7 +2466,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
@@ -2394,7 +2486,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>161</v>
       </c>
@@ -2411,6 +2503,26 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.93400000000000005</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -2420,13 +2532,13 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE323FF4-989B-4276-A839-D0FF7CE8EDDF}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="37.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>137</v>
       </c>
@@ -2434,7 +2546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -2454,7 +2566,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -2462,7 +2574,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -2482,7 +2594,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -2502,7 +2614,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -2522,7 +2634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -2542,7 +2654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -2550,7 +2662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2570,7 +2682,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -2590,7 +2702,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -2610,7 +2722,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -2630,7 +2742,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2650,7 +2762,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -2670,7 +2782,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -2690,7 +2802,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -2710,7 +2822,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
@@ -2730,7 +2842,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>161</v>
       </c>
@@ -2747,6 +2859,26 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.93400000000000005</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -2756,13 +2888,13 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2082DC88-DFF2-40CF-B4DF-7066E382B5F7}">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>138</v>
       </c>
@@ -2770,7 +2902,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -2790,7 +2922,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -2798,7 +2930,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -2818,7 +2950,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -2838,7 +2970,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -2856,7 +2988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -2874,7 +3006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -2882,7 +3014,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -2902,7 +3034,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -2922,7 +3054,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>25</v>
       </c>
@@ -2942,7 +3074,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>26</v>
       </c>
@@ -2962,7 +3094,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>27</v>
       </c>
@@ -2982,7 +3114,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>28</v>
       </c>
@@ -3002,7 +3134,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -3022,7 +3154,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>30</v>
       </c>
@@ -3042,7 +3174,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>31</v>
       </c>
@@ -3060,6 +3192,46 @@
       <c r="F17">
         <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
         <v>0.98</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="B18" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C18">
+        <f>VLOOKUP(B18, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F18">
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>48</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.99199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3069,14 +3241,14 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF7280D3-4B67-4A70-8D20-99496E68EF3A}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="23.85546875" customWidth="1"/>
     <col min="6" max="6" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>141</v>
       </c>
@@ -3084,7 +3256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -3104,7 +3276,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="7" t="s">
         <v>144</v>
       </c>
@@ -3112,7 +3284,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>60</v>
       </c>
@@ -3131,7 +3303,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>61</v>
       </c>
@@ -3150,7 +3322,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>27</v>
       </c>
@@ -3170,7 +3342,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -3190,7 +3362,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="B8" t="s">
         <v>2</v>
       </c>
@@ -3210,7 +3382,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>25</v>
       </c>
@@ -3230,7 +3402,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>26</v>
       </c>
@@ -3250,7 +3422,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>162</v>
       </c>
@@ -3267,6 +3439,26 @@
       <c r="F11">
         <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="B12" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C12">
+        <f>VLOOKUP(B12, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F12">
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -3276,13 +3468,13 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22ACFE10-4BB6-46C8-8EC7-C9A1D50150CB}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>142</v>
       </c>
@@ -3290,7 +3482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -3310,7 +3502,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="7" t="s">
         <v>144</v>
       </c>
@@ -3318,7 +3510,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>60</v>
       </c>
@@ -3335,7 +3527,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>61</v>
       </c>
@@ -3354,7 +3546,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>27</v>
       </c>
@@ -3374,7 +3566,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -3394,7 +3586,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="B8" t="s">
         <v>2</v>
       </c>
@@ -3414,7 +3606,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>25</v>
       </c>
@@ -3434,7 +3626,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>26</v>
       </c>
@@ -3454,7 +3646,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>162</v>
       </c>
@@ -3471,6 +3663,26 @@
       <c r="F11">
         <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="B12" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C12">
+        <f>VLOOKUP(B12, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F12">
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -3480,13 +3692,13 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6749F6D7-861C-4875-81CE-3B633F4D2DE8}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>140</v>
       </c>
@@ -3494,7 +3706,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -3514,7 +3726,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="7" t="s">
         <v>143</v>
       </c>
@@ -3522,7 +3734,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>60</v>
       </c>
@@ -3539,7 +3751,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>61</v>
       </c>
@@ -3558,7 +3770,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>27</v>
       </c>
@@ -3578,7 +3790,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -3598,7 +3810,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="B8" t="s">
         <v>2</v>
       </c>
@@ -3618,7 +3830,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>25</v>
       </c>
@@ -3638,7 +3850,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>26</v>
       </c>
@@ -3658,7 +3870,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>160</v>
       </c>
@@ -3675,6 +3887,46 @@
       <c r="F11">
         <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$2:$G$48,3,FALSE)</f>
         <v>0.89400000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="B12" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C12">
+        <f>VLOOKUP(B12, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F12">
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="B13" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C13">
+        <f>VLOOKUP(B13, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>48</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="F13">
+        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.99199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3686,18 +3938,18 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82B0CCBA-0AAC-49C1-B314-C4A1ABA2F1AC}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.140625" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -3717,7 +3969,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -3725,7 +3977,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -3745,7 +3997,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -3765,7 +4017,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -3783,7 +4035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -3801,7 +4053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -3809,7 +4061,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -3829,7 +4081,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -3849,7 +4101,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>25</v>
       </c>
@@ -3869,7 +4121,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>26</v>
       </c>
@@ -3889,7 +4141,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>27</v>
       </c>
@@ -3909,7 +4161,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>28</v>
       </c>
@@ -3929,7 +4181,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -3949,7 +4201,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>30</v>
       </c>
@@ -3969,7 +4221,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>31</v>
       </c>
@@ -3989,7 +4241,47 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
+      <c r="B18" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C18">
+        <f>VLOOKUP(B18, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F18">
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>48</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.99199999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6">
       <c r="B21" s="2"/>
     </row>
   </sheetData>
@@ -3999,13 +4291,13 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C43C1D89-69F4-4A96-941A-67F76960DD3E}">
-  <dimension ref="A1:B47"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B49"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="116" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4013,7 +4305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -4021,7 +4313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -4029,7 +4321,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -4037,7 +4329,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -4045,7 +4337,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -4053,7 +4345,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -4061,7 +4353,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -4069,7 +4361,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>63</v>
       </c>
@@ -4077,7 +4369,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -4085,7 +4377,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -4093,7 +4385,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -4101,7 +4393,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -4109,7 +4401,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -4117,7 +4409,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -4125,7 +4417,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -4133,7 +4425,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -4141,7 +4433,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>59</v>
       </c>
@@ -4149,7 +4441,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -4157,7 +4449,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -4165,7 +4457,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -4173,7 +4465,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -4181,7 +4473,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>31</v>
       </c>
@@ -4189,7 +4481,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2">
       <c r="A24" t="s">
         <v>48</v>
       </c>
@@ -4197,7 +4489,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2">
       <c r="A25" t="s">
         <v>51</v>
       </c>
@@ -4205,7 +4497,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -4213,7 +4505,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2">
       <c r="A27" t="s">
         <v>49</v>
       </c>
@@ -4221,7 +4513,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -4229,7 +4521,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -4237,7 +4529,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2">
       <c r="A30" t="s">
         <v>52</v>
       </c>
@@ -4245,7 +4537,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2">
       <c r="A31" t="s">
         <v>39</v>
       </c>
@@ -4253,7 +4545,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -4261,7 +4553,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2">
       <c r="A33" t="s">
         <v>27</v>
       </c>
@@ -4269,7 +4561,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -4277,7 +4569,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2">
       <c r="A35" t="s">
         <v>25</v>
       </c>
@@ -4285,7 +4577,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2">
       <c r="A36" t="s">
         <v>3</v>
       </c>
@@ -4293,7 +4585,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2">
       <c r="A37" t="s">
         <v>26</v>
       </c>
@@ -4301,7 +4593,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2">
       <c r="A38" t="s">
         <v>64</v>
       </c>
@@ -4309,7 +4601,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2">
       <c r="A39" t="s">
         <v>53</v>
       </c>
@@ -4317,7 +4609,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -4325,7 +4617,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2">
       <c r="A41" t="s">
         <v>2</v>
       </c>
@@ -4333,7 +4625,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2">
       <c r="A42" t="s">
         <v>60</v>
       </c>
@@ -4341,7 +4633,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2">
       <c r="A43" t="s">
         <v>61</v>
       </c>
@@ -4349,7 +4641,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2">
       <c r="A44" t="s">
         <v>62</v>
       </c>
@@ -4357,7 +4649,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2">
       <c r="A45" t="s">
         <v>160</v>
       </c>
@@ -4365,7 +4657,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2">
       <c r="A46" t="s">
         <v>161</v>
       </c>
@@ -4373,12 +4665,28 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2">
       <c r="A47" t="s">
         <v>162</v>
       </c>
       <c r="B47">
         <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B48">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B49">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -4388,8 +4696,8 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27EE3377-032C-4CE0-A3B7-5FFD545CF0F5}">
-  <dimension ref="A1:P49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P50"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" customWidth="1"/>
@@ -4655,7 +4963,7 @@
     <col min="16134" max="16135" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
@@ -4692,7 +5000,7 @@
       <c r="N1" s="15"/>
       <c r="O1" s="15"/>
     </row>
-    <row r="2" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -4733,7 +5041,7 @@
       </c>
       <c r="O2" s="28"/>
     </row>
-    <row r="3" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="45">
       <c r="A3" t="s">
         <v>72</v>
       </c>
@@ -4780,7 +5088,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
         <v>74</v>
       </c>
@@ -4823,7 +5131,7 @@
       <c r="N4" s="17"/>
       <c r="O4" s="17"/>
     </row>
-    <row r="5" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="30">
       <c r="A5" t="s">
         <v>75</v>
       </c>
@@ -4866,7 +5174,7 @@
       <c r="N5" s="18"/>
       <c r="O5" s="18"/>
     </row>
-    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="30">
       <c r="A6" t="s">
         <v>76</v>
       </c>
@@ -4911,7 +5219,7 @@
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="25.5">
       <c r="A7" t="s">
         <v>79</v>
       </c>
@@ -4956,7 +5264,7 @@
       <c r="N7" s="11"/>
       <c r="O7" s="11"/>
     </row>
-    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="30">
       <c r="A8" t="s">
         <v>80</v>
       </c>
@@ -5003,7 +5311,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="30">
       <c r="A9" t="s">
         <v>82</v>
       </c>
@@ -5050,7 +5358,7 @@
         <v>95.9</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="45">
       <c r="A10" t="s">
         <v>84</v>
       </c>
@@ -5093,7 +5401,7 @@
       <c r="N10" s="19"/>
       <c r="O10" s="19"/>
     </row>
-    <row r="11" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="30">
       <c r="A11" t="s">
         <v>86</v>
       </c>
@@ -5136,7 +5444,7 @@
       <c r="N11" s="20"/>
       <c r="O11" s="20"/>
     </row>
-    <row r="12" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="30">
       <c r="A12" t="s">
         <v>88</v>
       </c>
@@ -5179,7 +5487,7 @@
       <c r="N12" s="21"/>
       <c r="O12" s="21"/>
     </row>
-    <row r="13" spans="1:15" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="63.75">
       <c r="A13" t="s">
         <v>90</v>
       </c>
@@ -5224,7 +5532,7 @@
       <c r="N13" s="20"/>
       <c r="O13" s="20"/>
     </row>
-    <row r="14" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="60">
       <c r="A14" t="s">
         <v>93</v>
       </c>
@@ -5267,7 +5575,7 @@
       <c r="N14" s="19"/>
       <c r="O14" s="19"/>
     </row>
-    <row r="15" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="60">
       <c r="A15" t="s">
         <v>94</v>
       </c>
@@ -5310,7 +5618,7 @@
       <c r="N15" s="20"/>
       <c r="O15" s="20"/>
     </row>
-    <row r="16" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="60">
       <c r="A16" t="s">
         <v>95</v>
       </c>
@@ -5355,7 +5663,7 @@
       <c r="N16" s="19"/>
       <c r="O16" s="19"/>
     </row>
-    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="30">
       <c r="A17" t="s">
         <v>97</v>
       </c>
@@ -5401,7 +5709,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="45">
       <c r="A18" t="s">
         <v>98</v>
       </c>
@@ -5444,7 +5752,7 @@
       <c r="N18" s="19"/>
       <c r="O18" s="19"/>
     </row>
-    <row r="19" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="45">
       <c r="A19" t="s">
         <v>99</v>
       </c>
@@ -5491,7 +5799,7 @@
       <c r="N19" s="20"/>
       <c r="O19" s="20"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16">
       <c r="A20" t="s">
         <v>101</v>
       </c>
@@ -5524,7 +5832,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="60">
       <c r="A21" t="s">
         <v>103</v>
       </c>
@@ -5555,7 +5863,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="60">
       <c r="A22" t="s">
         <v>104</v>
       </c>
@@ -5586,7 +5894,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="60">
       <c r="A23" t="s">
         <v>105</v>
       </c>
@@ -5617,7 +5925,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="60">
       <c r="A24" t="s">
         <v>106</v>
       </c>
@@ -5648,7 +5956,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16">
       <c r="A25" t="s">
         <v>108</v>
       </c>
@@ -5677,7 +5985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16">
       <c r="A26" t="s">
         <v>109</v>
       </c>
@@ -5706,7 +6014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16">
       <c r="A27" t="s">
         <v>110</v>
       </c>
@@ -5735,7 +6043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16">
       <c r="A28" t="s">
         <v>111</v>
       </c>
@@ -5764,7 +6072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" ht="45">
       <c r="A29" t="s">
         <v>112</v>
       </c>
@@ -5795,7 +6103,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" ht="30">
       <c r="A30" t="s">
         <v>113</v>
       </c>
@@ -5824,7 +6132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16">
       <c r="A31" t="s">
         <v>114</v>
       </c>
@@ -5853,7 +6161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16">
       <c r="A32" t="s">
         <v>115</v>
       </c>
@@ -5882,7 +6190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>116</v>
       </c>
@@ -5911,7 +6219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>117</v>
       </c>
@@ -5942,7 +6250,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" ht="30">
       <c r="A35" t="s">
         <v>119</v>
       </c>
@@ -5973,7 +6281,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>121</v>
       </c>
@@ -6004,7 +6312,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="30">
       <c r="A37" t="s">
         <v>123</v>
       </c>
@@ -6035,7 +6343,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>124</v>
       </c>
@@ -6066,7 +6374,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="30">
       <c r="A39" t="s">
         <v>125</v>
       </c>
@@ -6097,7 +6405,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>126</v>
       </c>
@@ -6126,7 +6434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
         <v>127</v>
       </c>
@@ -6159,7 +6467,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9">
       <c r="A42" t="s">
         <v>128</v>
       </c>
@@ -6192,7 +6500,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
         <v>130</v>
       </c>
@@ -6220,7 +6528,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="45">
       <c r="A44" t="s">
         <v>131</v>
       </c>
@@ -6251,7 +6559,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
         <v>132</v>
       </c>
@@ -6279,7 +6587,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9">
       <c r="A46" t="s">
         <v>168</v>
       </c>
@@ -6309,7 +6617,7 @@
         <v>0.89400000000000002</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9">
       <c r="A47" t="s">
         <v>167</v>
       </c>
@@ -6339,7 +6647,7 @@
         <v>0.93400000000000005</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9">
       <c r="A48" t="s">
         <v>166</v>
       </c>
@@ -6367,9 +6675,57 @@
         <v>0.84</v>
       </c>
     </row>
-    <row r="49" spans="8:9" x14ac:dyDescent="0.25">
-      <c r="H49" s="25"/>
-      <c r="I49" s="25"/>
+    <row r="49" spans="1:9">
+      <c r="A49" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B49" s="4">
+        <v>47</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F49" s="30">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="G49" s="30">
+        <v>0.97599999999999998</v>
+      </c>
+      <c r="H49" s="30">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="I49" s="30">
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B50" s="4">
+        <v>48</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F50" s="30">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="G50" s="30">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="H50" s="30">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="I50" s="30">
+        <v>0.99199999999999999</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6383,13 +6739,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45FA39FB-289A-4CDC-A78E-AD026F2859AE}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="116" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -6397,7 +6753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -6417,7 +6773,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -6425,7 +6781,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -6437,15 +6793,15 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.64</v>
       </c>
       <c r="F4">
-        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B4,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -6457,15 +6813,15 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.75</v>
       </c>
       <c r="F5">
-        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B5,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -6477,13 +6833,15 @@
         <v>0</v>
       </c>
       <c r="E6">
+        <f>VLOOKUP(B6,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>1</v>
       </c>
       <c r="F6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <f>VLOOKUP(B6,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -6495,13 +6853,15 @@
         <v>0</v>
       </c>
       <c r="E7">
+        <f>VLOOKUP(B7,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>1</v>
       </c>
       <c r="F7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <f>VLOOKUP(B7,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -6509,184 +6869,224 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
       <c r="C9">
-        <f>VLOOKUP(B9, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B9, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>39</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9">
-        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
-        <v>0.84</v>
+        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
+        <v>0.76400000000000001</v>
       </c>
       <c r="F9">
-        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
-        <v>0.97</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <f>VLOOKUP(B9,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
+        <v>0.99199999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
       <c r="C10">
-        <f>VLOOKUP(B10, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B10, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>40</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
-        <v>0.84</v>
+        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
+        <v>0.76400000000000001</v>
       </c>
       <c r="F10">
-        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
-        <v>0.97</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <f>VLOOKUP(B10,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
+        <v>0.99199999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>25</v>
       </c>
       <c r="C11">
-        <f>VLOOKUP(B11, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B11, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>34</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.73</v>
       </c>
       <c r="F11">
-        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B11,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>26</v>
       </c>
       <c r="C12">
-        <f>VLOOKUP(B12, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B12, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>36</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.8</v>
       </c>
       <c r="F12">
-        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B12,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>27</v>
       </c>
       <c r="C13">
-        <f>VLOOKUP(B13, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B13, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>32</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.84099999999999997</v>
       </c>
       <c r="F13">
-        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B13,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>28</v>
       </c>
       <c r="C14">
-        <f>VLOOKUP(B14, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B14, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>19</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14">
-        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.93</v>
       </c>
       <c r="F14">
-        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B14,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>29</v>
       </c>
       <c r="C15">
-        <f>VLOOKUP(B15, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B15, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>20</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.93</v>
       </c>
       <c r="F15">
-        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B15,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>30</v>
       </c>
       <c r="C16">
-        <f>VLOOKUP(B16, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B16, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>21</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.93</v>
       </c>
       <c r="F16">
-        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B16,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>31</v>
       </c>
       <c r="C17">
-        <f>VLOOKUP(B17, IDs!$A$1:$B$44,2, FALSE)</f>
+        <f>VLOOKUP(B17, IDs!$A$1:$B$50,2, FALSE)</f>
         <v>22</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$G$45,2,TRUE)</f>
+        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$G$50,2,TRUE)</f>
         <v>0.93</v>
       </c>
       <c r="F17">
-        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
+        <f>VLOOKUP(B17,DiagnosisSensAndSpec!$E$1:$G$50,3,TRUE)</f>
         <v>0.98</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="B18" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C18">
+        <f>VLOOKUP(B18, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F18">
+        <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>48</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.99199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -6697,13 +7097,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0F64AF9-9ECE-4E3E-A2D1-05BE152A0480}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="101.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -6711,7 +7111,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -6731,7 +7131,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -6739,7 +7139,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -6759,7 +7159,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -6779,7 +7179,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -6799,7 +7199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -6819,7 +7219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -6827,7 +7227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -6847,7 +7247,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -6867,7 +7267,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -6887,7 +7287,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -6907,7 +7307,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -6927,7 +7327,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -6947,7 +7347,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -6967,7 +7367,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -6987,7 +7387,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
@@ -7007,7 +7407,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>162</v>
       </c>
@@ -7024,6 +7424,26 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.84</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -7033,13 +7453,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DC60C1E-2CE2-467A-895F-DEF1211E8D04}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="101.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -7047,7 +7467,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -7067,7 +7487,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -7075,7 +7495,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -7095,7 +7515,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -7115,7 +7535,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -7135,7 +7555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -7155,7 +7575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -7163,7 +7583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -7183,7 +7603,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -7203,7 +7623,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -7223,7 +7643,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -7243,7 +7663,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -7263,7 +7683,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -7283,7 +7703,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -7303,7 +7723,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -7323,7 +7743,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
@@ -7343,7 +7763,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>162</v>
       </c>
@@ -7360,6 +7780,26 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.84</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -7369,13 +7809,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F3293F-5A17-4180-BF24-E430C8DADB1C}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>35</v>
       </c>
@@ -7383,7 +7823,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -7403,7 +7843,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -7411,7 +7851,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -7431,7 +7871,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -7451,7 +7891,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -7469,7 +7909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -7487,7 +7927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -7495,7 +7935,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -7515,7 +7955,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -7535,7 +7975,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>25</v>
       </c>
@@ -7555,7 +7995,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>26</v>
       </c>
@@ -7575,7 +8015,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>27</v>
       </c>
@@ -7595,7 +8035,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>28</v>
       </c>
@@ -7615,7 +8055,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -7635,7 +8075,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>30</v>
       </c>
@@ -7655,7 +8095,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>31</v>
       </c>
@@ -7675,7 +8115,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>160</v>
       </c>
@@ -7692,6 +8132,46 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$2:$G$48,3,FALSE)</f>
         <v>0.89400000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C20">
+        <f>VLOOKUP(B20, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>48</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <f>VLOOKUP(B20,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="F20">
+        <f>VLOOKUP(B20,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.99199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -7701,13 +8181,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{775DE79B-3AB1-4B9D-8C6D-1BAB88363D05}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="101.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -7715,7 +8195,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -7735,7 +8215,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -7743,7 +8223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -7763,7 +8243,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -7783,7 +8263,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -7803,7 +8283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -7823,7 +8303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -7831,7 +8311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -7851,7 +8331,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -7871,7 +8351,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -7891,7 +8371,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -7911,7 +8391,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -7931,7 +8411,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -7951,7 +8431,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -7971,7 +8451,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -7991,7 +8471,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
@@ -8011,7 +8491,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>161</v>
       </c>
@@ -8028,6 +8508,26 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.93400000000000005</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -8037,13 +8537,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EA6C606-720F-4288-A97A-19A60E6C9529}">
-  <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="51.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -8051,7 +8551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -8071,7 +8571,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -8079,7 +8579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -8099,7 +8599,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -8119,7 +8619,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -8137,7 +8637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -8155,7 +8655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -8163,7 +8663,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>39</v>
       </c>
@@ -8183,7 +8683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>40</v>
       </c>
@@ -8203,7 +8703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>41</v>
       </c>
@@ -8223,7 +8723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>42</v>
       </c>
@@ -8243,7 +8743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>43</v>
       </c>
@@ -8263,7 +8763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>44</v>
       </c>
@@ -8283,7 +8783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>45</v>
       </c>
@@ -8303,7 +8803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>46</v>
       </c>
@@ -8323,7 +8823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="B17" t="s">
         <v>47</v>
       </c>
@@ -8343,7 +8843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="B18" t="s">
         <v>48</v>
       </c>
@@ -8363,7 +8863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="B19" t="s">
         <v>49</v>
       </c>
@@ -8383,7 +8883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="B20" t="s">
         <v>50</v>
       </c>
@@ -8403,7 +8903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="B21" t="s">
         <v>51</v>
       </c>
@@ -8423,7 +8923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="B22" t="s">
         <v>52</v>
       </c>
@@ -8443,7 +8943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="B23" t="s">
         <v>53</v>
       </c>
@@ -8463,7 +8963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -8471,7 +8971,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7">
       <c r="B25" t="s">
         <v>1</v>
       </c>
@@ -8491,7 +8991,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7">
       <c r="B26" t="s">
         <v>2</v>
       </c>
@@ -8509,6 +9009,46 @@
       <c r="F26">
         <f>VLOOKUP(B26,DiagnosisSensAndSpec!$E$1:$G$45,3,TRUE)</f>
         <v>0.97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="B27" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C27">
+        <f>VLOOKUP(B27, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <f>VLOOKUP(B27,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F27">
+        <f>VLOOKUP(B27,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.97599999999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="B28" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C28">
+        <f>VLOOKUP(B28, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>48</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <f>VLOOKUP(B28,DiagnosisSensAndSpec!$E$1:$I$50,2,FALSE)</f>
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="F28">
+        <f>VLOOKUP(B28,DiagnosisSensAndSpec!$E$1:$I$50,3,FALSE)</f>
+        <v>0.99199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -8518,13 +9058,13 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F86C481-A3CC-447D-99ED-82C53BDA94EE}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="101.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>54</v>
       </c>
@@ -8532,7 +9072,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -8552,7 +9092,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -8560,7 +9100,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -8580,7 +9120,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -8600,7 +9140,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -8620,7 +9160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -8640,7 +9180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -8648,7 +9188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -8668,7 +9208,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -8688,7 +9228,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -8708,7 +9248,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -8728,7 +9268,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -8748,7 +9288,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -8768,7 +9308,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -8788,7 +9328,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -8808,7 +9348,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
@@ -8828,7 +9368,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>162</v>
       </c>
@@ -8845,6 +9385,26 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.84</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -8855,13 +9415,13 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B59A441-0D38-4F1B-81D6-EE728C64E62D}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="101.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -8869,7 +9429,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -8889,7 +9449,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -8897,7 +9457,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -8917,7 +9477,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="B5" t="s">
         <v>15</v>
       </c>
@@ -8937,7 +9497,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -8957,7 +9517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -8977,7 +9537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -8985,7 +9545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -9005,7 +9565,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="B10" t="s">
         <v>2</v>
       </c>
@@ -9025,7 +9585,7 @@
         <v>0.95900000000000007</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -9045,7 +9605,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="B12" t="s">
         <v>64</v>
       </c>
@@ -9065,7 +9625,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -9085,7 +9645,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -9105,7 +9665,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -9125,7 +9685,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="B16" t="s">
         <v>7</v>
       </c>
@@ -9145,7 +9705,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" t="s">
         <v>8</v>
       </c>
@@ -9165,7 +9725,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" t="s">
         <v>162</v>
       </c>
@@ -9182,6 +9742,26 @@
       <c r="F18">
         <f>VLOOKUP(B18,DiagnosisSensAndSpec!$E$1:$I$48,5,FALSE)</f>
         <v>0.84</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19">
+        <f>VLOOKUP(B19, IDs!$A$1:$B$50,2, FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,4,FALSE)</f>
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="F19">
+        <f>VLOOKUP(B19,DiagnosisSensAndSpec!$E$1:$I$50,5,FALSE)</f>
+        <v>0.97599999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>